<commit_message>
Added placeholders to schedule
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/guiliberali/Library/Mobile Documents/com~apple~CloudDocs/Teaching /Teaching - BigData/Teach_BigData 2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/guiliberali/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B8B5798-C910-044E-8D21-D32AAE337C5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D54323-5439-5443-AB6A-F3BCF6EDA303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17480" xr2:uid="{16787138-0C24-184A-98B2-327E13C17B03}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
   <si>
     <t>Monday</t>
   </si>
@@ -159,6 +159,15 @@
   </si>
   <si>
     <t>UCB, Contextual, Fairness</t>
+  </si>
+  <si>
+    <t>Placeholder 1</t>
+  </si>
+  <si>
+    <t>Placeholder 2</t>
+  </si>
+  <si>
+    <t>By mid-august we will know if we will use this date</t>
   </si>
 </sst>
 </file>
@@ -661,12 +670,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="2" width="7.83203125" style="2" customWidth="1"/>
-    <col min="3" max="5" width="15.5" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.5" style="2" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" style="2" customWidth="1"/>
     <col min="6" max="6" width="42.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -987,6 +998,52 @@
         <v>27</v>
       </c>
     </row>
+    <row r="29" spans="2:7" ht="22" x14ac:dyDescent="0.3">
+      <c r="B29" s="4">
+        <v>42</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="10"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="22" x14ac:dyDescent="0.3">
+      <c r="B30" s="2">
+        <v>42</v>
+      </c>
+      <c r="C30" s="8"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+    </row>
+    <row r="31" spans="2:7" ht="22" x14ac:dyDescent="0.3">
+      <c r="B31" s="2">
+        <v>42</v>
+      </c>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G31" s="16"/>
+    </row>
+    <row r="32" spans="2:7" ht="22" x14ac:dyDescent="0.3">
+      <c r="B32" s="3">
+        <v>42</v>
+      </c>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="13"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="75" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>